<commit_message>
chore: sync workspace changes
</commit_message>
<xml_diff>
--- a/quotation/询价模版.xlsx
+++ b/quotation/询价模版.xlsx
@@ -67,6 +67,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>几个</t>
     </r>
     <r>
@@ -90,6 +96,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量</t>
     </r>
     <r>
@@ -104,6 +116,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量</t>
     </r>
     <r>
@@ -118,6 +136,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量</t>
     </r>
     <r>
@@ -132,6 +156,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量</t>
     </r>
     <r>
@@ -146,6 +176,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量</t>
     </r>
     <r>
@@ -160,6 +196,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户报价</t>
     </r>
     <r>
@@ -174,6 +216,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户报价</t>
     </r>
     <r>
@@ -188,6 +236,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户报价</t>
     </r>
     <r>
@@ -202,6 +256,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户报价</t>
     </r>
     <r>
@@ -216,6 +276,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户报价</t>
     </r>
     <r>
@@ -233,6 +299,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>长</t>
     </r>
     <r>
@@ -247,6 +319,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>宽</t>
     </r>
     <r>
@@ -261,6 +339,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>高</t>
     </r>
     <r>
@@ -278,6 +362,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>件数</t>
     </r>
     <r>
@@ -307,6 +397,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@</t>
     </r>
     <r>
@@ -348,6 +444,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@</t>
     </r>
     <r>
@@ -389,6 +491,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@</t>
     </r>
     <r>
@@ -430,6 +538,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@</t>
     </r>
     <r>
@@ -498,6 +612,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@</t>
     </r>
     <r>
@@ -533,6 +653,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>产品采购单价</t>
     </r>
     <r>
@@ -559,6 +685,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial Regular"/>
+        <charset val="134"/>
+      </rPr>
       <t>@1688</t>
     </r>
     <r>
@@ -687,6 +819,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利</t>
     </r>
     <r>
@@ -701,6 +839,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利率</t>
     </r>
     <r>
@@ -715,6 +859,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利率</t>
     </r>
     <r>
@@ -729,6 +879,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利率</t>
     </r>
     <r>
@@ -743,6 +899,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利率</t>
     </r>
     <r>
@@ -757,6 +919,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF262626"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>毛利率</t>
     </r>
     <r>
@@ -792,6 +960,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>红色</t>
     </r>
     <r>
@@ -874,6 +1048,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
       <t>例如开模费</t>
     </r>
     <r>
@@ -897,6 +1077,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="宋体-简"/>
+        <charset val="134"/>
+      </rPr>
       <t>客户需求量下方的计费重量如果低于</t>
     </r>
     <r>
@@ -991,7 +1177,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="13">
+  <numFmts count="14">
+    <numFmt numFmtId="26" formatCode="\$#,##0.00_);[Red]\(\$#,##0.00\)"/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
@@ -2261,8 +2448,8 @@
     <xf numFmtId="182" fontId="19" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="26" fontId="26" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2974,15 +3161,15 @@
         <v>54</v>
       </c>
       <c r="B17" s="41">
-        <f>MAX(B16,$G9)</f>
+        <f>MAX(B16,$G9/1000)</f>
         <v>0</v>
       </c>
       <c r="C17" s="41">
-        <f>MAX(C16,$G9)</f>
+        <f>MAX(C16,$G9/1000)</f>
         <v>0</v>
       </c>
       <c r="D17" s="66">
-        <f>MAX(D16,$G9)</f>
+        <f>MAX(D16,$G9/1000)</f>
         <v>0</v>
       </c>
       <c r="E17" s="63" t="s">
@@ -3184,19 +3371,19 @@
         <f>IF(B4&lt;&gt;"",($B$23+B$7)*B$4,"")</f>
         <v/>
       </c>
-      <c r="G23" s="77" t="str">
+      <c r="G23" s="69" t="str">
         <f>IF(C4&lt;&gt;"",($B$23+C$7)*C$4,"")</f>
         <v/>
       </c>
-      <c r="H23" s="77" t="str">
+      <c r="H23" s="69" t="str">
         <f>IF(D4&lt;&gt;"",($B$23+D$7)*D$4,"")</f>
         <v/>
       </c>
-      <c r="I23" s="77" t="str">
+      <c r="I23" s="69" t="str">
         <f>IF(E4&lt;&gt;"",($B$23+E$7)*E$4,"")</f>
         <v/>
       </c>
-      <c r="J23" s="77" t="str">
+      <c r="J23" s="69" t="str">
         <f>IF(F4&lt;&gt;"",($B$23+F$7)*F$4,"")</f>
         <v/>
       </c>
@@ -3227,19 +3414,19 @@
         <f>IF(B4&lt;&gt;"",($C$23+B$7)*B$4,"")</f>
         <v/>
       </c>
-      <c r="G24" s="77" t="str">
+      <c r="G24" s="69" t="str">
         <f>IF(C4&lt;&gt;"",($C$23+C$7)*C$4,"")</f>
         <v/>
       </c>
-      <c r="H24" s="77" t="str">
+      <c r="H24" s="69" t="str">
         <f>IF(D4&lt;&gt;"",($C$23+D$7)*D$4,"")</f>
         <v/>
       </c>
-      <c r="I24" s="77" t="str">
+      <c r="I24" s="69" t="str">
         <f>IF(E4&lt;&gt;"",($C$23+E$7)*E$4,"")</f>
         <v/>
       </c>
-      <c r="J24" s="77" t="str">
+      <c r="J24" s="69" t="str">
         <f>IF(F4&lt;&gt;"",($C$23+F$7)*F$4,"")</f>
         <v/>
       </c>
@@ -3269,19 +3456,19 @@
         <f>IF(B4&lt;&gt;"",($D$23+B$7)*B$4,"")</f>
         <v/>
       </c>
-      <c r="G25" s="77" t="str">
+      <c r="G25" s="69" t="str">
         <f>IF(C4&lt;&gt;"",($D$23+C$7)*C$4,"")</f>
         <v/>
       </c>
-      <c r="H25" s="77" t="str">
+      <c r="H25" s="69" t="str">
         <f>IF(D4&lt;&gt;"",($D$23+D$7)*D$4,"")</f>
         <v/>
       </c>
-      <c r="I25" s="77" t="str">
+      <c r="I25" s="69" t="str">
         <f>IF(E4&lt;&gt;"",($D$23+E$7)*E$4,"")</f>
         <v/>
       </c>
-      <c r="J25" s="77" t="str">
+      <c r="J25" s="69" t="str">
         <f>IF(F4&lt;&gt;"",($D$23+F$7)*F$4,"")</f>
         <v/>
       </c>
@@ -3705,7 +3892,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="iconSet" priority="1" id="{739315a7-dcf0-4fcb-ab19-74775ac8c728}">
+          <x14:cfRule type="iconSet" priority="1" id="{deb92356-c951-4384-ad66-e9de75618911}">
             <x14:iconSet iconSet="3TrafficLights2" custom="1">
               <x14:cfvo type="percent">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
chore: sync workspace updates
</commit_message>
<xml_diff>
--- a/quotation/询价模版.xlsx
+++ b/quotation/询价模版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="12920"/>
+    <workbookView windowWidth="29400" windowHeight="12960"/>
   </bookViews>
   <sheets>
     <sheet name="报价表" sheetId="1" r:id="rId1"/>
@@ -2386,15 +2386,15 @@
         <v>56</v>
       </c>
       <c r="B18" s="70">
-        <f>IFERROR(B16/$G9,0)</f>
+        <f>IFERROR(B16/($G9/1000),0)</f>
         <v>0</v>
       </c>
       <c r="C18" s="70">
-        <f>IFERROR(C16/$G9,0)</f>
+        <f>IFERROR(C16/($G9/1000),0)</f>
         <v>0</v>
       </c>
       <c r="D18" s="71">
-        <f>IFERROR(D16/$G9,0)</f>
+        <f>IFERROR(D16/($G9/1000),0)</f>
         <v>0</v>
       </c>
       <c r="E18" s="62" t="s">

</xml_diff>